<commit_message>
Added code to write results in Excel file
</commit_message>
<xml_diff>
--- a/Defect_classification_project/Reference_keywords.xlsx
+++ b/Defect_classification_project/Reference_keywords.xlsx
@@ -19,12 +19,30 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Performance Keywords</t>
   </si>
   <si>
     <t>Performance</t>
+  </si>
+  <si>
+    <t>slowness</t>
+  </si>
+  <si>
+    <t>slow</t>
+  </si>
+  <si>
+    <t>responds slowly</t>
+  </si>
+  <si>
+    <t>loading issue</t>
+  </si>
+  <si>
+    <t>long load time</t>
+  </si>
+  <si>
+    <t>loading slowly</t>
   </si>
 </sst>
 </file>
@@ -357,7 +375,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
@@ -373,6 +391,36 @@
         <v>1</v>
       </c>
     </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Added code for getting jira description
</commit_message>
<xml_diff>
--- a/Defect_classification_project/Reference_keywords.xlsx
+++ b/Defect_classification_project/Reference_keywords.xlsx
@@ -19,10 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>Performance Keywords</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Performance</t>
   </si>
@@ -42,14 +39,56 @@
     <t>long load time</t>
   </si>
   <si>
-    <t>loading slowly</t>
+    <t>Loading slowness</t>
+  </si>
+  <si>
+    <t>time to render the complete page</t>
+  </si>
+  <si>
+    <t>time to render the page</t>
+  </si>
+  <si>
+    <t>response time</t>
+  </si>
+  <si>
+    <t>slow response</t>
+  </si>
+  <si>
+    <t>wait time</t>
+  </si>
+  <si>
+    <t>average load time</t>
+  </si>
+  <si>
+    <t>peak response time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">throughput </t>
+  </si>
+  <si>
+    <t>performance statistics</t>
+  </si>
+  <si>
+    <t>network profiling</t>
+  </si>
+  <si>
+    <t>Time taken</t>
+  </si>
+  <si>
+    <t>load</t>
+  </si>
+  <si>
+    <t>seconds</t>
+  </si>
+  <si>
+    <t>minutes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -57,27 +96,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -92,9 +117,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -375,50 +399,115 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
+      <c r="A1" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>